<commit_message>
Holiday printables: rename shop to Pantry Printable Co. (Etsy: PantryPrintableCo)
Owner picked the new shop name. Replaced the old name in every source, then
rebuilt all PDFs, the tracker .xlsx, listing images, pins and the Thanksgiving
bundle files, and refreshed the 8 upload kits.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014RfnYfVJj2WjcFbtCk72fp
</commit_message>
<xml_diff>
--- a/downloads/holiday/gift-budget-tracker/1-files/Christmas-Gift-Budget-Tracker-Example.xlsx
+++ b/downloads/holiday/gift-budget-tracker/1-files/Christmas-Gift-Budget-Tracker-Example.xlsx
@@ -774,7 +774,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Quiet Table Co.  ·  Excel + Google Sheets  ·  Made for one household, for personal use</t>
+          <t>Pantry Printable Co.  ·  Excel + Google Sheets  ·  Made for one household, for personal use</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -931,7 +931,7 @@
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Merry Christmas from Quiet Table Co.</t>
+          <t>Merry Christmas from Pantry Printable Co.</t>
         </is>
       </c>
     </row>

</xml_diff>